<commit_message>
Rebuild size/variant axes: separate Size×Variant grid, 3-column import, disable invalid combos on PDP
- Importer: add `variants` + `stock_matrix` columns and parseStockMatrix
  (explicit size:variant:qty triples, no cartesian phantoms; legacy
  color|size:stock still parsed as fallback). DB field `color` unchanged.
- Admin editor: rename second axis to "Variant"; grid only exposes inputs
  for offered (size,variant) pairs, others render a clickable "—".
- PDP: per-(size,variant) stock resolution disables unavailable options
  given the current selection; customer-facing "Color" renamed to "Variant".
- Regenerate bulk-import templates + docs in lockstep.
</commit_message>
<xml_diff>
--- a/docs/bulk-import/MiniYo_Bulk_Import_Template.xlsx
+++ b/docs/bulk-import/MiniYo_Bulk_Import_Template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:Y4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -422,6 +422,8 @@
     <col min="21" max="21" width="12.83203125" customWidth="1"/>
     <col min="22" max="22" width="12.83203125" customWidth="1"/>
     <col min="23" max="23" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1"/>
+    <col min="25" max="25" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,6 +494,12 @@
         <v>sizes</v>
       </c>
       <c r="W1" t="str">
+        <v>variants</v>
+      </c>
+      <c r="X1" t="str">
+        <v>stock_matrix</v>
+      </c>
+      <c r="Y1" t="str">
         <v>images</v>
       </c>
     </row>
@@ -563,6 +571,12 @@
         <v>0-3M:5, 3-6M:8, 6-9M:3</v>
       </c>
       <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
         <v>SAMPLE-001_1.jpg, SAMPLE-001_2.jpg</v>
       </c>
     </row>
@@ -631,9 +645,15 @@
         <v>sleepwear,gift</v>
       </c>
       <c r="V3" t="str">
-        <v>Beige|0-3M:4, Beige|3-6M:2, Gray|0-3M:3</v>
+        <v>0-3M|3-6M</v>
       </c>
       <c r="W3" t="str">
+        <v>Beige|Gray</v>
+      </c>
+      <c r="X3" t="str">
+        <v>0-3M:Beige:4; 3-6M:Beige:2; 0-3M:Gray:3</v>
+      </c>
+      <c r="Y3" t="str">
         <v>SAMPLE-002_1.jpg</v>
       </c>
     </row>
@@ -705,12 +725,18 @@
         <v>One Size:8</v>
       </c>
       <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
         <v>https://example.com/sample-cap.jpg</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rebuild size/variant axes: separate Size×Variant grid, 3-column import, disable invalid combos on PDP (#31)
- Importer: add `variants` + `stock_matrix` columns and parseStockMatrix
  (explicit size:variant:qty triples, no cartesian phantoms; legacy
  color|size:stock still parsed as fallback). DB field `color` unchanged.
- Admin editor: rename second axis to "Variant"; grid only exposes inputs
  for offered (size,variant) pairs, others render a clickable "—".
- PDP: per-(size,variant) stock resolution disables unavailable options
  given the current selection; customer-facing "Color" renamed to "Variant".
- Regenerate bulk-import templates + docs in lockstep.

Co-authored-by: Omran Kassaa <omraniik@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/bulk-import/MiniYo_Bulk_Import_Template.xlsx
+++ b/docs/bulk-import/MiniYo_Bulk_Import_Template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:Y4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -422,6 +422,8 @@
     <col min="21" max="21" width="12.83203125" customWidth="1"/>
     <col min="22" max="22" width="12.83203125" customWidth="1"/>
     <col min="23" max="23" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1"/>
+    <col min="25" max="25" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,6 +494,12 @@
         <v>sizes</v>
       </c>
       <c r="W1" t="str">
+        <v>variants</v>
+      </c>
+      <c r="X1" t="str">
+        <v>stock_matrix</v>
+      </c>
+      <c r="Y1" t="str">
         <v>images</v>
       </c>
     </row>
@@ -563,6 +571,12 @@
         <v>0-3M:5, 3-6M:8, 6-9M:3</v>
       </c>
       <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
         <v>SAMPLE-001_1.jpg, SAMPLE-001_2.jpg</v>
       </c>
     </row>
@@ -631,9 +645,15 @@
         <v>sleepwear,gift</v>
       </c>
       <c r="V3" t="str">
-        <v>Beige|0-3M:4, Beige|3-6M:2, Gray|0-3M:3</v>
+        <v>0-3M|3-6M</v>
       </c>
       <c r="W3" t="str">
+        <v>Beige|Gray</v>
+      </c>
+      <c r="X3" t="str">
+        <v>0-3M:Beige:4; 3-6M:Beige:2; 0-3M:Gray:3</v>
+      </c>
+      <c r="Y3" t="str">
         <v>SAMPLE-002_1.jpg</v>
       </c>
     </row>
@@ -705,12 +725,18 @@
         <v>One Size:8</v>
       </c>
       <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
         <v>https://example.com/sample-cap.jpg</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>